<commit_message>
Update NBA PostPlanner exports for 2026-06-29
Binary xlsx files regenerated during pipeline session.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkRM4GbRQFrMmG2cw4thK5
</commit_message>
<xml_diff>
--- a/NBA/postplanner-imports/hh-postplanner-2026-06-29.xlsx
+++ b/NBA/postplanner-imports/hh-postplanner-2026-06-29.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>06/29/2026  11:56</t>
+          <t>06/29/2026  09:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -495,7 +495,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>06/29/2026  13:26</t>
+          <t>06/29/2026  11:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -510,7 +510,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>06/29/2026  14:56</t>
+          <t>06/29/2026  13:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06/29/2026  16:26</t>
+          <t>06/29/2026  16:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -540,7 +540,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06/29/2026  17:56</t>
+          <t>06/29/2026  19:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -555,7 +555,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/29/2026  19:26</t>
+          <t>06/29/2026  21:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>